<commit_message>
SFX, Music and background sprite refined
</commit_message>
<xml_diff>
--- a/assets/resources/reactii_final.xlsx
+++ b/assets/resources/reactii_final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25225"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\itfest-game\assets\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6959D4EC-06E1-4AF2-B01D-23ACC780BBF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F975D58C-BE4F-4E33-8BEA-A7D34458F77A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -294,7 +294,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -313,6 +313,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="18">
     <border>
@@ -555,7 +561,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -593,10 +599,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -622,9 +628,12 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -640,9 +649,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Стандартная">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -680,7 +689,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Стандартная">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -786,7 +795,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Стандартная">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -928,7 +937,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1343,7 +1352,7 @@
       <c r="F10" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="18" t="s">
+      <c r="G10" s="32" t="s">
         <v>41</v>
       </c>
       <c r="H10" s="11" t="s">
@@ -2227,6 +2236,6 @@
     <row r="25" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>